<commit_message>
Added no absent summary
</commit_message>
<xml_diff>
--- a/file_IX_Monday_student_data.xlsx
+++ b/file_IX_Monday_student_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\29abh\Projects\RAC_Projects\RACOperationalApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02DB7E30-51FD-42B4-A7C3-FBB77DFCA4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1372CB24-E1A1-46BD-8CDE-26B6F4D9E26D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="28800" windowHeight="15370" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Name</t>
   </si>
@@ -44,192 +44,6 @@
   </si>
   <si>
     <t>Roll Number</t>
-  </si>
-  <si>
-    <t>Aarav Kashyap</t>
-  </si>
-  <si>
-    <t>Aarav Mahajan</t>
-  </si>
-  <si>
-    <t>Abhigyan Kumar</t>
-  </si>
-  <si>
-    <t>Abir</t>
-  </si>
-  <si>
-    <t>Prithvi Singh</t>
-  </si>
-  <si>
-    <t>Agrim Bakshi</t>
-  </si>
-  <si>
-    <t>Anirudh Singh</t>
-  </si>
-  <si>
-    <t>Arnav Gupta</t>
-  </si>
-  <si>
-    <t>Aryan Raj</t>
-  </si>
-  <si>
-    <t>Atharv Kumar</t>
-  </si>
-  <si>
-    <t>Ayana Rana</t>
-  </si>
-  <si>
-    <t>Ayansh Rungta</t>
-  </si>
-  <si>
-    <t>Chamandeep Kaur</t>
-  </si>
-  <si>
-    <t>Dhriti</t>
-  </si>
-  <si>
-    <t>Priyanshi</t>
-  </si>
-  <si>
-    <t>Divisha Gupta</t>
-  </si>
-  <si>
-    <t>Kabir</t>
-  </si>
-  <si>
-    <t>Geetali Singh</t>
-  </si>
-  <si>
-    <t>Honeyka</t>
-  </si>
-  <si>
-    <t>Ishaan Gupta</t>
-  </si>
-  <si>
-    <t>Jai Patel</t>
-  </si>
-  <si>
-    <t>Janya Sharma</t>
-  </si>
-  <si>
-    <t>Jeetika</t>
-  </si>
-  <si>
-    <t>Jyena Ratra</t>
-  </si>
-  <si>
-    <t>Kaashvi</t>
-  </si>
-  <si>
-    <t>Kaasni</t>
-  </si>
-  <si>
-    <t>Kairav Jindal</t>
-  </si>
-  <si>
-    <t>Kavish Narwat</t>
-  </si>
-  <si>
-    <t>Yash Chaudhary</t>
-  </si>
-  <si>
-    <t>Kiana</t>
-  </si>
-  <si>
-    <t>Krisha</t>
-  </si>
-  <si>
-    <t>Manan</t>
-  </si>
-  <si>
-    <t>Krishiv Gandhi</t>
-  </si>
-  <si>
-    <t>Kriti</t>
-  </si>
-  <si>
-    <t>Kush Agarwal</t>
-  </si>
-  <si>
-    <t>Lakshay Tyagi</t>
-  </si>
-  <si>
-    <t>Manya</t>
-  </si>
-  <si>
-    <t>Maulik</t>
-  </si>
-  <si>
-    <t>Pratishtha Ahlawat</t>
-  </si>
-  <si>
-    <t>Mishika</t>
-  </si>
-  <si>
-    <t>Navika Pandey</t>
-  </si>
-  <si>
-    <t>Nishtha Kaul</t>
-  </si>
-  <si>
-    <t>Pranay Bansal</t>
-  </si>
-  <si>
-    <t>Peevaree</t>
-  </si>
-  <si>
-    <t>Reet Narula</t>
-  </si>
-  <si>
-    <t>Rian</t>
-  </si>
-  <si>
-    <t>Aryaman</t>
-  </si>
-  <si>
-    <t>Mishika Ahuja</t>
-  </si>
-  <si>
-    <t>Rishita Dahiya</t>
-  </si>
-  <si>
-    <t>Shaivee</t>
-  </si>
-  <si>
-    <t>Shambhavi Gupta</t>
-  </si>
-  <si>
-    <t>Shubham Gupta</t>
-  </si>
-  <si>
-    <t>Smriddhi</t>
-  </si>
-  <si>
-    <t>Kashvi</t>
-  </si>
-  <si>
-    <t>Saumya</t>
-  </si>
-  <si>
-    <t>Swastika</t>
-  </si>
-  <si>
-    <t>Tanmay Tyagi</t>
-  </si>
-  <si>
-    <t>Uddhav Sharma</t>
-  </si>
-  <si>
-    <t>Vihan Jhwar</t>
-  </si>
-  <si>
-    <t>Riddhi</t>
-  </si>
-  <si>
-    <t>Yahaana Rao</t>
-  </si>
-  <si>
-    <t>Yukti</t>
   </si>
 </sst>
 </file>
@@ -623,508 +437,256 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="3">
-        <v>919560299662</v>
-      </c>
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
     </row>
     <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="3">
-        <v>919873793777</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="3">
-        <v>919582942729</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="3"/>
     </row>
     <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="3">
-        <v>919315993446</v>
-      </c>
+      <c r="A5" s="2"/>
+      <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="3">
-        <v>919540090026</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="3"/>
     </row>
     <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="3">
-        <v>919999190354</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="B7" s="3"/>
     </row>
     <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="3">
-        <v>919873553300</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="3"/>
     </row>
     <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="3">
-        <v>919910460002</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="3"/>
     </row>
     <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="3">
-        <v>919560601943</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="3">
-        <v>919643164987</v>
-      </c>
+      <c r="A11" s="2"/>
+      <c r="B11" s="3"/>
     </row>
     <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="3">
-        <v>918130280411</v>
-      </c>
+      <c r="A12" s="2"/>
+      <c r="B12" s="3"/>
     </row>
     <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="3">
-        <v>919717273628</v>
-      </c>
+      <c r="A13" s="2"/>
+      <c r="B13" s="3"/>
     </row>
     <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="3">
-        <v>919899789468</v>
-      </c>
+      <c r="A14" s="2"/>
+      <c r="B14" s="3"/>
     </row>
     <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="3">
-        <v>919005262222</v>
-      </c>
+      <c r="A15" s="2"/>
+      <c r="B15" s="3"/>
     </row>
     <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="3">
-        <v>918130532126</v>
-      </c>
+      <c r="A16" s="2"/>
+      <c r="B16" s="3"/>
     </row>
     <row r="17" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="3">
-        <v>919971007310</v>
-      </c>
+      <c r="A17" s="2"/>
+      <c r="B17" s="3"/>
     </row>
     <row r="18" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="3">
-        <v>919958309190</v>
-      </c>
+      <c r="A18" s="2"/>
+      <c r="B18" s="3"/>
     </row>
     <row r="19" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="3">
-        <v>919810931501</v>
-      </c>
+      <c r="A19" s="2"/>
+      <c r="B19" s="3"/>
     </row>
     <row r="20" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="3">
-        <v>918447706950</v>
-      </c>
+      <c r="A20" s="2"/>
+      <c r="B20" s="3"/>
     </row>
     <row r="21" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="3">
-        <v>919810405656</v>
-      </c>
+      <c r="A21" s="2"/>
+      <c r="B21" s="3"/>
     </row>
     <row r="22" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="3">
-        <v>919891611780</v>
-      </c>
+      <c r="A22" s="2"/>
+      <c r="B22" s="3"/>
     </row>
     <row r="23" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="3">
-        <v>918295218151</v>
-      </c>
+      <c r="A23" s="2"/>
+      <c r="B23" s="3"/>
     </row>
     <row r="24" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" s="3">
-        <v>919650295091</v>
-      </c>
+      <c r="A24" s="2"/>
+      <c r="B24" s="3"/>
     </row>
     <row r="25" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B25" s="3">
-        <v>919161073999</v>
-      </c>
+      <c r="A25" s="2"/>
+      <c r="B25" s="3"/>
     </row>
     <row r="26" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" s="3">
-        <v>919210881660</v>
-      </c>
+      <c r="A26" s="2"/>
+      <c r="B26" s="3"/>
     </row>
     <row r="27" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="3">
-        <v>918448129927</v>
-      </c>
+      <c r="A27" s="2"/>
+      <c r="B27" s="3"/>
     </row>
     <row r="28" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="3">
-        <v>919899770356</v>
-      </c>
+      <c r="A28" s="2"/>
+      <c r="B28" s="3"/>
     </row>
     <row r="29" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B29" s="3">
-        <v>919953393534</v>
-      </c>
+      <c r="A29" s="2"/>
+      <c r="B29" s="3"/>
     </row>
     <row r="30" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B30" s="3">
-        <v>919717963357</v>
-      </c>
+      <c r="A30" s="2"/>
+      <c r="B30" s="3"/>
     </row>
     <row r="31" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" s="3">
-        <v>917678469620</v>
-      </c>
+      <c r="A31" s="2"/>
+      <c r="B31" s="3"/>
     </row>
     <row r="32" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B32" s="3">
-        <v>917676219891</v>
-      </c>
+      <c r="A32" s="2"/>
+      <c r="B32" s="3"/>
     </row>
     <row r="33" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B33" s="3">
-        <v>919212551204</v>
-      </c>
+      <c r="A33" s="2"/>
+      <c r="B33" s="3"/>
     </row>
     <row r="34" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="3">
-        <v>919999068676</v>
-      </c>
+      <c r="A34" s="2"/>
+      <c r="B34" s="3"/>
     </row>
     <row r="35" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B35" s="3">
-        <v>919718680678</v>
-      </c>
+      <c r="A35" s="2"/>
+      <c r="B35" s="3"/>
     </row>
     <row r="36" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B36" s="3">
-        <v>919717523005</v>
-      </c>
+      <c r="A36" s="2"/>
+      <c r="B36" s="3"/>
     </row>
     <row r="37" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B37" s="3">
-        <v>919891246558</v>
-      </c>
+      <c r="A37" s="2"/>
+      <c r="B37" s="3"/>
     </row>
     <row r="38" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B38" s="3">
-        <v>919899426612</v>
-      </c>
+      <c r="A38" s="2"/>
+      <c r="B38" s="3"/>
     </row>
     <row r="39" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" s="3">
-        <v>919910279520</v>
-      </c>
+      <c r="A39" s="2"/>
+      <c r="B39" s="3"/>
     </row>
     <row r="40" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B40" s="3">
-        <v>919871168342</v>
-      </c>
+      <c r="A40" s="2"/>
+      <c r="B40" s="3"/>
     </row>
     <row r="41" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B41" s="3">
-        <v>917838499469</v>
-      </c>
+      <c r="A41" s="2"/>
+      <c r="B41" s="3"/>
     </row>
     <row r="42" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B42" s="3">
-        <v>919717001371</v>
-      </c>
+      <c r="A42" s="2"/>
+      <c r="B42" s="3"/>
     </row>
     <row r="43" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B43" s="3">
-        <v>919899887554</v>
-      </c>
+      <c r="A43" s="2"/>
+      <c r="B43" s="3"/>
     </row>
     <row r="44" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B44" s="3">
-        <v>918901545656</v>
-      </c>
+      <c r="A44" s="2"/>
+      <c r="B44" s="3"/>
     </row>
     <row r="45" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A45" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B45" s="3">
-        <v>919873877907</v>
-      </c>
+      <c r="A45" s="2"/>
+      <c r="B45" s="3"/>
     </row>
     <row r="46" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A46" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B46" s="3">
-        <v>919811637600</v>
-      </c>
+      <c r="A46" s="2"/>
+      <c r="B46" s="3"/>
     </row>
     <row r="47" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A47" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B47" s="3">
-        <v>919871342496</v>
-      </c>
+      <c r="A47" s="2"/>
+      <c r="B47" s="3"/>
     </row>
     <row r="48" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A48" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B48" s="3">
-        <v>919911453881</v>
-      </c>
+      <c r="A48" s="2"/>
+      <c r="B48" s="3"/>
     </row>
     <row r="49" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A49" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49" s="3">
-        <v>919958302101</v>
-      </c>
+      <c r="A49" s="2"/>
+      <c r="B49" s="3"/>
     </row>
     <row r="50" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A50" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B50" s="3">
-        <v>919871354333</v>
-      </c>
+      <c r="A50" s="2"/>
+      <c r="B50" s="3"/>
     </row>
     <row r="51" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A51" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B51" s="3">
-        <v>919899506776</v>
-      </c>
+      <c r="A51" s="2"/>
+      <c r="B51" s="3"/>
     </row>
     <row r="52" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A52" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B52" s="3">
-        <v>919958244077</v>
-      </c>
+      <c r="A52" s="2"/>
+      <c r="B52" s="3"/>
     </row>
     <row r="53" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B53" s="3">
-        <v>919898490924</v>
-      </c>
+      <c r="A53" s="2"/>
+      <c r="B53" s="3"/>
     </row>
     <row r="54" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A54" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B54" s="3">
-        <v>918860634347</v>
-      </c>
+      <c r="A54" s="2"/>
+      <c r="B54" s="3"/>
     </row>
     <row r="55" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A55" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B55" s="3">
-        <v>919871608396</v>
-      </c>
+      <c r="A55" s="2"/>
+      <c r="B55" s="3"/>
     </row>
     <row r="56" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A56" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B56" s="3">
-        <v>918527796514</v>
-      </c>
+      <c r="A56" s="2"/>
+      <c r="B56" s="3"/>
     </row>
     <row r="57" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A57" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B57" s="3">
-        <v>919650522523</v>
-      </c>
+      <c r="A57" s="2"/>
+      <c r="B57" s="3"/>
     </row>
     <row r="58" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A58" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B58" s="3">
-        <v>918447700423</v>
-      </c>
+      <c r="A58" s="2"/>
+      <c r="B58" s="3"/>
     </row>
     <row r="59" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A59" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B59" s="3">
-        <v>918368945752</v>
-      </c>
+      <c r="A59" s="2"/>
+      <c r="B59" s="3"/>
     </row>
     <row r="60" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A60" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B60" s="3">
-        <v>919821775616</v>
-      </c>
+      <c r="A60" s="2"/>
+      <c r="B60" s="3"/>
     </row>
     <row r="61" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A61" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B61" s="3">
-        <v>919871622334</v>
-      </c>
+      <c r="A61" s="2"/>
+      <c r="B61" s="3"/>
     </row>
     <row r="62" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A62" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B62" s="3">
-        <v>919971988981</v>
-      </c>
+      <c r="A62" s="2"/>
+      <c r="B62" s="3"/>
     </row>
     <row r="63" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A63" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B63" s="3">
-        <v>919999017189</v>
-      </c>
+      <c r="A63" s="2"/>
+      <c r="B63" s="3"/>
     </row>
     <row r="64" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A64" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B64" s="3">
-        <v>919999174553</v>
-      </c>
+      <c r="A64" s="2"/>
+      <c r="B64" s="3"/>
     </row>
     <row r="65" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="2"/>

</xml_diff>

<commit_message>
Fixed some issues and added support for cloud xls sync
</commit_message>
<xml_diff>
--- a/file_IX_Monday_student_data.xlsx
+++ b/file_IX_Monday_student_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\29abh\Projects\RAC_Projects\RACOperationalApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1372CB24-E1A1-46BD-8CDE-26B6F4D9E26D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30950076-0B8C-4FF8-B407-03AE74769819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="28800" windowHeight="15370" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22540" yWindow="10430" windowWidth="14240" windowHeight="10450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Name</t>
   </si>
@@ -44,6 +44,12 @@
   </si>
   <si>
     <t>Roll Number</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>8, 9, 4, 3</t>
   </si>
 </sst>
 </file>
@@ -392,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.36328125" customWidth="1"/>
@@ -408,6 +414,17 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>